<commit_message>
Added the rest of deflection analysis, and updated time and notes on stats
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A2C2F8A-5B55-449A-90BE-9CDED4225AA9}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D0DF912-63A2-42C3-AD98-99F78B1AE77A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -18,7 +18,6 @@
     <sheet name="Concrete" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -156,6 +155,12 @@
   </si>
   <si>
     <t>Concrete Beams Deflection</t>
+  </si>
+  <si>
+    <t>might need to add a question for if flat roof since different equation for allowable deflection</t>
+  </si>
+  <si>
+    <t>Some reason the sys.exit() prints more don’t know why</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -1051,7 +1056,7 @@
         <v>2.5</v>
       </c>
       <c r="G2">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1127,6 +1132,14 @@
       <c r="D15" t="s">
         <v>34</v>
       </c>
+      <c r="G15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added Beam Design Known Dimensions flexure only, still needs shear and deflection, and added time and notes to stats
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D0DF912-63A2-42C3-AD98-99F78B1AE77A}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F24E9E22-12D4-4D32-892F-B1756CBD1DFE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="44">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -161,6 +161,15 @@
   </si>
   <si>
     <t>Some reason the sys.exit() prints more don’t know why</t>
+  </si>
+  <si>
+    <t>Desgin Concrete Beams Known Dimensions</t>
+  </si>
+  <si>
+    <t>Currently only Flexure still needs deflection and shear</t>
+  </si>
+  <si>
+    <t>Logic check required</t>
   </si>
 </sst>
 </file>
@@ -1003,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -1012,10 +1021,12 @@
     <col min="4" max="4" width="51.5546875" customWidth="1"/>
     <col min="5" max="5" width="14.88671875" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" customWidth="1"/>
+    <col min="7" max="7" width="72.109375" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4" t="s">
         <v>31</v>
@@ -1035,8 +1046,16 @@
       <c r="G1" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+    </row>
+    <row r="2" spans="1:13" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1058,8 +1077,11 @@
       <c r="G2">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
@@ -1069,63 +1091,63 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:7" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1135,10 +1157,16 @@
       <c r="G15" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="G16" t="s">
         <v>40</v>
+      </c>
+      <c r="H16" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some logic to calc Vu,Mu, and partial deflection for known beam, started shear desgin for known dimension beam but barely made a dent, and added time to stats
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F24E9E22-12D4-4D32-892F-B1756CBD1DFE}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1175D1A-9F4B-4143-B42B-0AA54D6C0B9F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>Logic check required</t>
+  </si>
+  <si>
+    <t>The \n not printing on the next line but being in the variable proprt</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -1078,7 +1081,7 @@
         <v>3.5</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1169,6 +1172,11 @@
         <v>42</v>
       </c>
     </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added point load shear desgin along with time to the stats.
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1175D1A-9F4B-4143-B42B-0AA54D6C0B9F}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{5DBB0EBC-E693-4F82-ACCD-31615A6E53F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2264B8E2-9CE7-475C-A0D3-634A06493BEF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t>The \n not printing on the next line but being in the variable proprt</t>
+  </si>
+  <si>
+    <t>Shear desgin for distributed isn't set up but point load is</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -1081,7 +1084,7 @@
         <v>3.5</v>
       </c>
       <c r="H2">
-        <v>5.75</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1177,6 +1180,11 @@
         <v>44</v>
       </c>
     </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
PM_interactionbase and further work on masonry column/wall computations.
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alisaleh/Desktop/Senior Collaborative Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEA3D89-25CF-CF4C-B94B-D2C7BD9743BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912C6927-B236-7742-8BA3-4908AA18469B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="27220" windowHeight="15040" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="53">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -188,6 +188,15 @@
   </si>
   <si>
     <t xml:space="preserve">Added tables for mortar strength, started column design file </t>
+  </si>
+  <si>
+    <t>Session 2</t>
+  </si>
+  <si>
+    <t>2hrs</t>
+  </si>
+  <si>
+    <t>Started developping PM interaction code for Column Design</t>
   </si>
 </sst>
 </file>
@@ -583,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5618AE-DEA8-4C1F-8212-87D46148B750}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
@@ -838,6 +847,17 @@
       </c>
       <c r="C27" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Started the Shear and Moment class to calc it fewer times in the code.
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alisaleh/Desktop/Senior Collaborative Project/Senior-Project-Code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BED34AD0-4A24-4556-8B9E-1BFA97841407}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="27220" windowHeight="15040" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
     <sheet name="Timber" sheetId="2" r:id="rId2"/>
     <sheet name="Concrete" sheetId="3" r:id="rId3"/>
+    <sheet name="Other" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="59">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -206,6 +207,15 @@
   </si>
   <si>
     <t>Completed Pn and Mn calcs for masonry + further masonry code</t>
+  </si>
+  <si>
+    <t>Shear and Moment Class</t>
+  </si>
+  <si>
+    <t>Point load needs a fix where it is both positive and negative, currently broken</t>
+  </si>
+  <si>
+    <t>Need to add a line at height 0 to orientate the beam</t>
   </si>
 </sst>
 </file>
@@ -602,14 +612,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5618AE-DEA8-4C1F-8212-87D46148B750}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.5" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
-    <col min="3" max="3" width="107.5" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" customWidth="1"/>
+    <col min="3" max="3" width="107.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -619,7 +629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" ht="21.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" s="1" customFormat="1" ht="21.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -631,7 +641,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
@@ -643,7 +653,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="1" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -655,7 +665,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="1" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -667,7 +677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
@@ -677,7 +687,7 @@
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
@@ -687,7 +697,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" s="1" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
@@ -697,7 +707,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -707,7 +717,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
@@ -717,7 +727,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" s="1" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
@@ -727,7 +737,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
@@ -737,7 +747,7 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
@@ -747,7 +757,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" s="1" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
@@ -757,43 +767,43 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="6"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>18</v>
       </c>
@@ -805,7 +815,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
@@ -815,7 +825,7 @@
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>23</v>
       </c>
@@ -825,7 +835,7 @@
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -833,13 +843,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>46</v>
       </c>
@@ -847,7 +857,7 @@
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>48</v>
       </c>
@@ -858,7 +868,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>50</v>
       </c>
@@ -869,7 +879,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>53</v>
       </c>
@@ -888,15 +898,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC543DE1-7AFB-4EBE-B969-1754C2BEFA61}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.6640625" customWidth="1"/>
     <col min="2" max="2" width="33.33203125" customWidth="1"/>
     <col min="3" max="3" width="75" customWidth="1"/>
-    <col min="4" max="4" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4" t="s">
         <v>26</v>
@@ -906,7 +916,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -918,7 +928,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
@@ -928,7 +938,7 @@
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -938,7 +948,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -948,7 +958,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
@@ -958,7 +968,7 @@
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
@@ -968,7 +978,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
@@ -978,7 +988,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -988,7 +998,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
@@ -998,7 +1008,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
@@ -1008,61 +1018,61 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>18</v>
       </c>
@@ -1080,20 +1090,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
   <dimension ref="A1:M18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.5" customWidth="1"/>
-    <col min="3" max="3" width="23.83203125" customWidth="1"/>
-    <col min="4" max="4" width="51.5" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="19.77734375" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
+    <col min="4" max="4" width="51.44140625" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>
-    <col min="7" max="7" width="72.1640625" customWidth="1"/>
+    <col min="7" max="7" width="72.109375" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="32.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4" t="s">
         <v>31</v>
@@ -1122,7 +1132,7 @@
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
-    <row r="2" spans="1:13" ht="16.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1148,7 +1158,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
@@ -1158,63 +1168,63 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:13" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="29.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:13" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="29.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:13" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1228,7 +1238,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="G16" t="s">
         <v>40</v>
       </c>
@@ -1236,14 +1246,102 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7982EEB8-C046-4557-A0F1-9E18C2D9AD96}">
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Seperated all of Concrete beams into own files
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BED34AD0-4A24-4556-8B9E-1BFA97841407}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF0BD98C-2BE9-4835-8ABB-E847008E4A24}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -216,6 +216,15 @@
   </si>
   <si>
     <t>Need to add a line at height 0 to orientate the beam</t>
+  </si>
+  <si>
+    <t>Desgin Concrete Beams unKnown Dimensions</t>
+  </si>
+  <si>
+    <t>Seperating into single files</t>
+  </si>
+  <si>
+    <t>Possibly Multi input is causing the problem</t>
   </si>
 </sst>
 </file>
@@ -292,6 +301,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1099,8 +1112,9 @@
     <col min="5" max="5" width="14.77734375" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>
     <col min="7" max="7" width="72.109375" customWidth="1"/>
-    <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="15.77734375" customWidth="1"/>
+    <col min="8" max="8" width="51" customWidth="1"/>
+    <col min="9" max="9" width="27.77734375" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="32.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1126,8 +1140,12 @@
       <c r="H1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="I1" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
@@ -1156,6 +1174,9 @@
       </c>
       <c r="H2">
         <v>7.75</v>
+      </c>
+      <c r="J2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1236,6 +1257,9 @@
       </c>
       <c r="H15" t="s">
         <v>43</v>
+      </c>
+      <c r="J15" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fixed The UI's to work
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF0BD98C-2BE9-4835-8ABB-E847008E4A24}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{719531BB-1805-4A56-AC05-5368EDE43F60}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Possibly Multi input is causing the problem</t>
+  </si>
+  <si>
+    <t>Fixing UI</t>
   </si>
 </sst>
 </file>
@@ -1287,75 +1290,87 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7982EEB8-C046-4557-A0F1-9E18C2D9AD96}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="2" max="2" width="60.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1363,7 +1378,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
Started disrributed shear design
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{719531BB-1805-4A56-AC05-5368EDE43F60}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BAD376D-1E9F-46E0-9BC9-51983A392DDB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -1176,7 +1176,7 @@
         <v>3.5</v>
       </c>
       <c r="H2">
-        <v>7.75</v>
+        <v>9.25</v>
       </c>
       <c r="J2">
         <v>0.5</v>

</xml_diff>

<commit_message>
Finished to my Knowledge Shear desgin for concrete beam
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BAD376D-1E9F-46E0-9BC9-51983A392DDB}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B97E6BD-D0E5-4CCE-98ED-18D0ED44266D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -304,10 +304,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1176,7 +1172,7 @@
         <v>3.5</v>
       </c>
       <c r="H2">
-        <v>9.25</v>
+        <v>10.75</v>
       </c>
       <c r="J2">
         <v>0.5</v>

</xml_diff>

<commit_message>
Added deflection to concrete design along with a final print of all working desgined beams and its info
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B97E6BD-D0E5-4CCE-98ED-18D0ED44266D}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07A45ADE-B0E8-45F1-A114-3E58ADB3E142}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -1172,7 +1172,7 @@
         <v>3.5</v>
       </c>
       <c r="H2">
-        <v>10.75</v>
+        <v>11.75</v>
       </c>
       <c r="J2">
         <v>0.5</v>

</xml_diff>

<commit_message>
Added unknown beam dimension calcs. and found that distributed shear is breaking, will redo all of shear calcs to try and fix
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07A45ADE-B0E8-45F1-A114-3E58ADB3E142}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B78905C-5C52-4030-8B73-C56308FC5EAA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -304,6 +304,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1174,6 +1178,9 @@
       <c r="H2">
         <v>11.75</v>
       </c>
+      <c r="I2">
+        <v>1.5</v>
+      </c>
       <c r="J2">
         <v>0.5</v>
       </c>
@@ -1185,6 +1192,9 @@
       <c r="B3" s="4"/>
       <c r="C3" s="1"/>
       <c r="F3">
+        <v>0.5</v>
+      </c>
+      <c r="H3">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Shear for concrete beams
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B78905C-5C52-4030-8B73-C56308FC5EAA}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E612377-C1F3-4EA2-8572-C2491BAF50AE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -173,12 +173,6 @@
     <t>Logic check required</t>
   </si>
   <si>
-    <t>The \n not printing on the next line but being in the variable proprt</t>
-  </si>
-  <si>
-    <t>Shear desgin for distributed isn't set up but point load is</t>
-  </si>
-  <si>
     <t>Ali</t>
   </si>
   <si>
@@ -228,6 +222,9 @@
   </si>
   <si>
     <t>Fixing UI</t>
+  </si>
+  <si>
+    <t>Need to fix deflection calcs</t>
   </si>
 </sst>
 </file>
@@ -867,7 +864,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -875,35 +872,35 @@
     </row>
     <row r="27" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B27" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" t="s">
         <v>47</v>
-      </c>
-      <c r="C27" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" t="s">
         <v>50</v>
-      </c>
-      <c r="B28" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" t="s">
         <v>53</v>
-      </c>
-      <c r="B29" t="s">
-        <v>54</v>
-      </c>
-      <c r="C29" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1144,10 +1141,10 @@
         <v>41</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
@@ -1195,7 +1192,7 @@
         <v>0.5</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1268,7 +1265,7 @@
         <v>43</v>
       </c>
       <c r="J15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -1279,14 +1276,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H17" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1305,10 +1297,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1381,12 +1373,12 @@
         <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made Deflection work for unknown dimensions properly and started fixing when designs dont work and how it is displayed
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E612377-C1F3-4EA2-8572-C2491BAF50AE}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5001E4CF-024A-4748-B9E2-C2A510EFC363}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Need to fix deflection calcs</t>
+  </si>
+  <si>
+    <t>making the desgins work together</t>
   </si>
 </sst>
 </file>
@@ -301,10 +304,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1114,7 +1113,8 @@
     <col min="7" max="7" width="72.109375" customWidth="1"/>
     <col min="8" max="8" width="51" customWidth="1"/>
     <col min="9" max="9" width="27.77734375" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="10" max="10" width="33.88671875" customWidth="1"/>
+    <col min="11" max="11" width="17.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="32.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1146,7 +1146,9 @@
       <c r="J1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="4"/>
+      <c r="K1" s="4" t="s">
+        <v>62</v>
+      </c>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
@@ -1193,6 +1195,9 @@
       </c>
       <c r="H3">
         <v>2.5</v>
+      </c>
+      <c r="K3">
+        <v>1.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Shear checks added to stop it if not to code, only have deflection left and then better print
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5001E4CF-024A-4748-B9E2-C2A510EFC363}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EC14E4C-3235-4BBA-A12E-4AB25D597FD9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -304,6 +304,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1197,7 +1201,7 @@
         <v>2.5</v>
       </c>
       <c r="K3">
-        <v>1.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added end system for if no deflection works.
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EC14E4C-3235-4BBA-A12E-4AB25D597FD9}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A51EFD5C-A546-4FFE-B575-7794C2CAEEB1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -1201,7 +1201,7 @@
         <v>2.5</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Better Print System in place for concrete beam design
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A51EFD5C-A546-4FFE-B575-7794C2CAEEB1}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D03AB1F-A261-4F4C-9ABB-5EE7D8705E5E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -304,10 +304,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1201,7 +1197,7 @@
         <v>2.5</v>
       </c>
       <c r="K3">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Started doing hand calc comparision for time stats and check math of code
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D03AB1F-A261-4F4C-9ABB-5EE7D8705E5E}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0870145-5A13-41E2-A8F1-A706E3DC0C1B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="64">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -228,6 +228,9 @@
   </si>
   <si>
     <t>making the desgins work together</t>
+  </si>
+  <si>
+    <t>Calc 3 code time (mins)</t>
   </si>
 </sst>
 </file>
@@ -304,6 +307,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1218,43 +1225,72 @@
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="4">
+        <v>0.5</v>
+      </c>
       <c r="C6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="4">
+        <v>3</v>
+      </c>
       <c r="C7" s="1"/>
     </row>
     <row r="8" spans="1:13" ht="29.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="4">
+        <f>28.48/60</f>
+        <v>0.47466666666666668</v>
+      </c>
       <c r="C8" s="1"/>
     </row>
     <row r="9" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1"/>
+      <c r="B9" s="1">
+        <v>0.5</v>
+      </c>
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:13" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1"/>
+      <c r="B10" s="1">
+        <v>2</v>
+      </c>
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1"/>
+      <c r="B11" s="1">
+        <f>26.46/60</f>
+        <v>0.441</v>
+      </c>
       <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">

</xml_diff>

<commit_message>
More hand calcs to get time comparision and check for errors
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0870145-5A13-41E2-A8F1-A706E3DC0C1B}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CABD2488-AF15-4B53-B908-5905062FE746}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -1228,7 +1228,9 @@
       <c r="B6" s="4">
         <v>0.5</v>
       </c>
-      <c r="C6" s="1"/>
+      <c r="C6" s="4">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -1237,7 +1239,9 @@
       <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C7" s="1"/>
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" spans="1:13" ht="29.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
@@ -1247,7 +1251,10 @@
         <f>28.48/60</f>
         <v>0.47466666666666668</v>
       </c>
-      <c r="C8" s="1"/>
+      <c r="C8" s="1">
+        <f>28.03/60</f>
+        <v>0.46716666666666667</v>
+      </c>
     </row>
     <row r="9" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -1281,15 +1288,26 @@
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="B12">
+        <f>20/60</f>
+        <v>0.33333333333333331</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>63</v>
+      </c>
+      <c r="B14">
+        <f>20.98/60</f>
+        <v>0.34966666666666668</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
More hand calcs to compare and fixed printing errors
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CABD2488-AF15-4B53-B908-5905062FE746}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0A4ED00-5726-45C1-BA40-976609FE4EAB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="67">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -231,6 +231,15 @@
   </si>
   <si>
     <t>Calc 3 code time (mins)</t>
+  </si>
+  <si>
+    <t>Math run Notes</t>
+  </si>
+  <si>
+    <t>As was having infinte decimal so had to use round to fix</t>
+  </si>
+  <si>
+    <t>Notes while coding</t>
   </si>
 </sst>
 </file>
@@ -1108,12 +1117,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5F9580-F39B-450E-8581-0BC34D974670}">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.77734375" customWidth="1"/>
     <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" customWidth="1"/>
+    <col min="3" max="3" width="44.109375" customWidth="1"/>
     <col min="4" max="4" width="51.44140625" customWidth="1"/>
     <col min="5" max="5" width="14.77734375" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>
@@ -1263,7 +1272,9 @@
       <c r="B9" s="1">
         <v>0.5</v>
       </c>
-      <c r="C9" s="1"/>
+      <c r="C9" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="10" spans="1:13" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -1272,7 +1283,9 @@
       <c r="B10" s="1">
         <v>2</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
@@ -1282,7 +1295,10 @@
         <f>26.46/60</f>
         <v>0.441</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1">
+        <f>32.6/60</f>
+        <v>0.54333333333333333</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -1292,6 +1308,10 @@
         <f>20/60</f>
         <v>0.33333333333333331</v>
       </c>
+      <c r="C12">
+        <f>20/60</f>
+        <v>0.33333333333333331</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
@@ -1300,6 +1320,9 @@
       <c r="B13">
         <v>1</v>
       </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
     </row>
     <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
@@ -1309,10 +1332,14 @@
         <f>20.98/60</f>
         <v>0.34966666666666668</v>
       </c>
+      <c r="C14">
+        <f>26.25/60</f>
+        <v>0.4375</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D15" t="s">
         <v>34</v>
@@ -1335,9 +1362,17 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more trials and working on upgrades for loading of beam
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF005729-F7E4-4A70-A93A-9B1955385AFB}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E87C8F74-38E4-466A-9EAB-06D9E68B9ED0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="113">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -367,6 +367,18 @@
   </si>
   <si>
     <t>Concrte deflectio problem might be a messed up if statement for if beam has compressive steel.</t>
+  </si>
+  <si>
+    <t>Milan Chhetri</t>
+  </si>
+  <si>
+    <t>EE</t>
+  </si>
+  <si>
+    <t>This is awesome</t>
+  </si>
+  <si>
+    <t>Good calculations</t>
   </si>
 </sst>
 </file>
@@ -1609,7 +1621,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F03E159-22CD-4944-B0AB-9B6794C0D9B6}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1846,6 +1858,38 @@
         <v>107</v>
       </c>
     </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>111</v>
+      </c>
+      <c r="I8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J8" t="s">
+        <v>107</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changed times to be in minutes for hand calcs
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E87C8F74-38E4-466A-9EAB-06D9E68B9ED0}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87331B86-8041-4D27-B2B9-9C63865AF255}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="115">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -90,9 +90,6 @@
     <t>0.5 min for code 3 total to transfer</t>
   </si>
   <si>
-    <t>Hand Calc 3 time (hrs)</t>
-  </si>
-  <si>
     <t>Hand Calc 3 mistakes</t>
   </si>
   <si>
@@ -379,6 +376,15 @@
   </si>
   <si>
     <t>Good calculations</t>
+  </si>
+  <si>
+    <t>Hand Calc 1 time (mins)</t>
+  </si>
+  <si>
+    <t>Hand Calc 2 time (mins)</t>
+  </si>
+  <si>
+    <t>Hand Calc 3 time (mins)</t>
   </si>
 </sst>
 </file>
@@ -844,12 +850,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>8</v>
+        <v>112</v>
       </c>
       <c r="B6" s="5">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -874,12 +880,12 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="B9" s="5">
-        <v>0.75</v>
+        <v>45</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -904,19 +910,19 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="B12" s="5">
-        <v>0.75</v>
+        <v>45</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="5">
         <v>6</v>
@@ -972,32 +978,32 @@
     </row>
     <row r="21" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>24</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -1007,7 +1013,7 @@
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1018,7 +1024,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1026,35 +1032,35 @@
     </row>
     <row r="27" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" t="s">
         <v>46</v>
-      </c>
-      <c r="B27" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" t="s">
         <v>48</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>49</v>
-      </c>
-      <c r="C28" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
         <v>51</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>52</v>
-      </c>
-      <c r="C29" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1076,11 +1082,11 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1150,7 +1156,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -1180,7 +1186,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1241,10 +1247,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -1259,7 +1265,7 @@
   <dimension ref="A1:M19"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="24.44140625" customWidth="1"/>
     <col min="3" max="3" width="44.109375" customWidth="1"/>
     <col min="4" max="4" width="51.44140625" customWidth="1"/>
@@ -1275,34 +1281,34 @@
     <row r="1" spans="1:13" ht="32.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="K1" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
@@ -1371,13 +1377,13 @@
     </row>
     <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>8</v>
+        <v>112</v>
       </c>
       <c r="B6" s="4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="C6" s="4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1406,13 +1412,13 @@
     </row>
     <row r="9" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="B9" s="1">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="C9" s="1">
-        <v>0.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
@@ -1441,20 +1447,18 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="B12">
-        <f>20/60</f>
-        <v>0.33333333333333331</v>
+        <v>20</v>
       </c>
       <c r="C12">
-        <f>20/60</f>
-        <v>0.33333333333333331</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1465,7 +1469,7 @@
     </row>
     <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14">
         <f>20.98/60</f>
@@ -1478,40 +1482,40 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="G16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" t="s">
         <v>64</v>
-      </c>
-      <c r="C19" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1530,10 +1534,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1603,15 +1607,15 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1636,51 +1640,51 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" t="s">
         <v>67</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>70</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>71</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>72</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>73</v>
       </c>
-      <c r="I1" t="s">
-        <v>74</v>
-      </c>
       <c r="J1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
         <v>76</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" t="s">
         <v>77</v>
       </c>
-      <c r="C2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>78</v>
-      </c>
-      <c r="E2" t="s">
-        <v>79</v>
       </c>
       <c r="F2">
         <v>9.8000000000000007</v>
@@ -1689,30 +1693,30 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I2" t="s">
         <v>80</v>
       </c>
-      <c r="I2" t="s">
-        <v>81</v>
-      </c>
       <c r="J2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" t="s">
         <v>84</v>
       </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" t="s">
         <v>78</v>
-      </c>
-      <c r="E3" t="s">
-        <v>79</v>
       </c>
       <c r="F3">
         <v>8.8000000000000007</v>
@@ -1721,30 +1725,30 @@
         <v>10</v>
       </c>
       <c r="H3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" t="s">
         <v>86</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>87</v>
-      </c>
-      <c r="J3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
         <v>89</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>90</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
         <v>91</v>
-      </c>
-      <c r="D4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E4" t="s">
-        <v>92</v>
       </c>
       <c r="F4">
         <v>9.9</v>
@@ -1753,30 +1757,30 @@
         <v>9.8000000000000007</v>
       </c>
       <c r="H4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" t="s">
         <v>93</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>94</v>
-      </c>
-      <c r="J4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" t="s">
         <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" t="s">
-        <v>97</v>
       </c>
       <c r="F5">
         <v>7.5</v>
@@ -1785,30 +1789,30 @@
         <v>9</v>
       </c>
       <c r="H5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" t="s">
         <v>100</v>
-      </c>
-      <c r="B6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" t="s">
-        <v>101</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -1817,30 +1821,30 @@
         <v>9.5</v>
       </c>
       <c r="H6" t="s">
+        <v>101</v>
+      </c>
+      <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="I6" t="s">
-        <v>103</v>
-      </c>
       <c r="J6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7">
         <v>9</v>
@@ -1849,30 +1853,30 @@
         <v>10</v>
       </c>
       <c r="H7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I7" t="s">
         <v>105</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>106</v>
-      </c>
-      <c r="J7" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
         <v>109</v>
       </c>
-      <c r="B8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" t="s">
-        <v>110</v>
-      </c>
       <c r="E8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F8">
         <v>10</v>
@@ -1881,13 +1885,13 @@
         <v>10</v>
       </c>
       <c r="H8" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" t="s">
         <v>111</v>
       </c>
-      <c r="I8" t="s">
-        <v>112</v>
-      </c>
       <c r="J8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Have bases for the new beam loads figured out, now need to set up all required info to fully get all lengths.
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DFC387D-2C1F-41A5-907D-22A71D3931C2}"/>
+  <xr:revisionPtr revIDLastSave="229" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C067E1E9-F647-4855-B440-875569AE26F9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="124">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -406,6 +406,12 @@
   </si>
   <si>
     <t>Check Mu and Mcr limits for code.</t>
+  </si>
+  <si>
+    <t>Looked through what np has to offer and found append: which combines two arrays together. Sort: which sorts the elements in an array from least to largest. Unique: which removes any duplicate numbers.</t>
+  </si>
+  <si>
+    <t>Above note will be used to fix problems with the overlap of point loads.</t>
   </si>
 </sst>
 </file>
@@ -1546,7 +1552,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7982EEB8-C046-4557-A0F1-9E18C2D9AD96}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -1566,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1637,6 +1643,16 @@
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Working on getting shear to work with new x line of beam, still not working
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C067E1E9-F647-4855-B440-875569AE26F9}"/>
+  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF946D3-DBAB-4B2E-83A6-9E8D8579518F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
@@ -1572,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
       <c r="C2">
         <v>0</v>

</xml_diff>

<commit_message>
Beam Loading is know able to do point loads for moment and almost distributed, Still want to test distributed more
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Code_Project/Senior-Project-Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF946D3-DBAB-4B2E-83A6-9E8D8579518F}"/>
+  <xr:revisionPtr revIDLastSave="232" documentId="13_ncr:1_{03D5E261-7105-FB43-B709-E120BAE8085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29370073-B6F4-44D0-B5D6-B99ACC50E80F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D4ADAE51-B09C-407E-8FCD-E420C17C7471}"/>
   </bookViews>
   <sheets>
     <sheet name="Masonry" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="125">
   <si>
     <t>Masonry lintel/beam Analysis</t>
   </si>
@@ -412,6 +412,9 @@
   </si>
   <si>
     <t>Above note will be used to fix problems with the overlap of point loads.</t>
+  </si>
+  <si>
+    <t>The display is nice, I would include a simple nicely formated summary at the end with beam sizes, demand and capacity</t>
   </si>
 </sst>
 </file>
@@ -1982,8 +1985,14 @@
       <c r="F10">
         <v>7</v>
       </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
       <c r="H10" t="s">
         <v>120</v>
+      </c>
+      <c r="I10" t="s">
+        <v>124</v>
       </c>
       <c r="J10" t="s">
         <v>121</v>

</xml_diff>